<commit_message>
R1 - Partial Rep - In-text numbers not replicated, missing libraries, data cits, wrong readme title
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/econ0763/Downloads/JPE/JPE-Biasi-20220349/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8390E1A-4ADB-6640-822D-2BEAB4902A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="198">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -36,6 +36,75 @@
     <t>Reproduced?</t>
   </si>
   <si>
+    <t>synthetic_data/code/make_simulated_data.do</t>
+  </si>
+  <si>
+    <t>synthetic_data/raw WDPI-style synthetic inputs</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>code/master_synth.do</t>
+  </si>
+  <si>
+    <t>Synthetic data build driver</t>
+  </si>
+  <si>
+    <t>code/build/oldteacher_roster_build.do; staff_build.do; teachers_build.do; teachers_panel.do</t>
+  </si>
+  <si>
+    <t>Teacher roster/staff/panel files</t>
+  </si>
+  <si>
+    <t>code/build/va_teacherside_build.do; testscores_build.do</t>
+  </si>
+  <si>
+    <t>Test-score and teacher-side VA input files</t>
+  </si>
+  <si>
+    <t>code/build/valueadded_calculation*.do</t>
+  </si>
+  <si>
+    <t>Teacher value-added/contribution files</t>
+  </si>
+  <si>
+    <t>code/build/teachers_with_allva.do</t>
+  </si>
+  <si>
+    <t>Final teacher panel with value-added</t>
+  </si>
+  <si>
+    <t>code/build/schedule_new.do; gen_omegas*.do</t>
+  </si>
+  <si>
+    <t>Wage schedule and omega input files</t>
+  </si>
+  <si>
+    <t>code/build/build_model_dataset*.do; build_teachers_offer_set.do</t>
+  </si>
+  <si>
+    <t>Model-estimation datasets</t>
+  </si>
+  <si>
+    <t>code/auxiliary_regressions/*.do</t>
+  </si>
+  <si>
+    <t>Auxiliary model moments for Fortran</t>
+  </si>
+  <si>
+    <t>code/build/omega_databuild.do; budget_overtime.do; build_distance_matrix.do; build_wageschedule_exitentry.do; fix_estsample_age.do</t>
+  </si>
+  <si>
+    <t>Model support files</t>
+  </si>
+  <si>
+    <t>code/build/build_model_dataset_pre2011.do; build_simulation_lndist.do</t>
+  </si>
+  <si>
+    <t>Pre-Act 10 simulation files</t>
+  </si>
+  <si>
     <t>Figure/Table #</t>
   </si>
   <si>
@@ -45,7 +114,511 @@
     <t>Line Number</t>
   </si>
   <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>code/descriptives/summary.do</t>
+  </si>
+  <si>
+    <t>15; 55</t>
+  </si>
+  <si>
+    <t>yes*</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t>code/auxiliary_regressions/aux_model_teachers_wages.do</t>
+  </si>
+  <si>
+    <t>285</t>
+  </si>
+  <si>
+    <t>Table 3</t>
+  </si>
+  <si>
+    <t>325; 335; 342</t>
+  </si>
+  <si>
+    <t>Table 4</t>
+  </si>
+  <si>
+    <t>code/descriptives/omega_analysis.do</t>
+  </si>
+  <si>
+    <t>101</t>
+  </si>
+  <si>
+    <t>Table 5</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_5_Table_A1.do</t>
+  </si>
+  <si>
+    <t>221</t>
+  </si>
+  <si>
+    <t>Table 6</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_6.do</t>
+  </si>
+  <si>
+    <t>272</t>
+  </si>
+  <si>
+    <t>Table 7</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_7.do</t>
+  </si>
+  <si>
+    <t>248</t>
+  </si>
+  <si>
+    <t>Table 8</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_8.do</t>
+  </si>
+  <si>
+    <t>178</t>
+  </si>
+  <si>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>code/descriptives/data_patterns.do</t>
+  </si>
+  <si>
+    <t>74</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>94; 164</t>
+  </si>
+  <si>
+    <t>Figure 3</t>
+  </si>
+  <si>
+    <t>231</t>
+  </si>
+  <si>
+    <t>Figure 4</t>
+  </si>
+  <si>
+    <t>code/descriptives/Figure_4.do</t>
+  </si>
+  <si>
+    <t>97</t>
+  </si>
+  <si>
+    <t>Table A1</t>
+  </si>
+  <si>
+    <t>Table A2</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_A2.do</t>
+  </si>
+  <si>
+    <t>112</t>
+  </si>
+  <si>
+    <t>Table A3</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_A3_PanelA.do; code/descriptives/Table_A3_PanelB.do</t>
+  </si>
+  <si>
+    <t>114; 50</t>
+  </si>
+  <si>
+    <t>Table B1</t>
+  </si>
+  <si>
+    <t>code/build/valueadded_calculation.do</t>
+  </si>
+  <si>
+    <t>250</t>
+  </si>
+  <si>
+    <t>Table B2</t>
+  </si>
+  <si>
+    <t>code/descriptives/appendix_figures.do</t>
+  </si>
+  <si>
+    <t>191</t>
+  </si>
+  <si>
+    <t>Table B3</t>
+  </si>
+  <si>
+    <t>code/descriptives/rothstein_test.do</t>
+  </si>
+  <si>
+    <t>241</t>
+  </si>
+  <si>
+    <t>Table B4</t>
+  </si>
+  <si>
+    <t>code/build/valueadded_calculation_classmodel.do</t>
+  </si>
+  <si>
+    <t>269</t>
+  </si>
+  <si>
+    <t>Table B5</t>
+  </si>
+  <si>
+    <t>code/auxiliary_regressions/auxmodels_teachers_varobust.do</t>
+  </si>
+  <si>
+    <t>327</t>
+  </si>
+  <si>
+    <t>Table B6</t>
+  </si>
+  <si>
+    <t>No standalone replication script</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Table B7</t>
+  </si>
+  <si>
+    <t>code/descriptives/c1c2_variation_studentlevel.do</t>
+  </si>
+  <si>
+    <t>192</t>
+  </si>
+  <si>
+    <t>Table B8</t>
+  </si>
+  <si>
+    <t>code/descriptives/achievement_race.do</t>
+  </si>
+  <si>
+    <t>185</t>
+  </si>
+  <si>
+    <t>Table B9</t>
+  </si>
+  <si>
+    <t>code/descriptives/schedule_summary.do</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>Table B10</t>
+  </si>
+  <si>
+    <t>code/descriptives/salary_variation.do</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>Table B11</t>
+  </si>
+  <si>
+    <t>code/auxiliary_regressions/auxiliary_models_teachers_info.do</t>
+  </si>
+  <si>
+    <t>203</t>
+  </si>
+  <si>
+    <t>Table B12</t>
+  </si>
+  <si>
+    <t>code/auxiliary_regressions/auxiliary_models_teachers_nobottom.do</t>
+  </si>
+  <si>
+    <t>304</t>
+  </si>
+  <si>
+    <t>Table B13</t>
+  </si>
+  <si>
+    <t>code/auxiliary_regressions/auxiliary_models_teachers_richprefs.do</t>
+  </si>
+  <si>
+    <t>69; 256</t>
+  </si>
+  <si>
+    <t>Table B14</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B14.do</t>
+  </si>
+  <si>
+    <t>3; 126</t>
+  </si>
+  <si>
+    <t>Table B15</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B15.do</t>
+  </si>
+  <si>
+    <t>1; 126</t>
+  </si>
+  <si>
+    <t>Table B16</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B16.do</t>
+  </si>
+  <si>
+    <t>Table B17</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B17.do</t>
+  </si>
+  <si>
+    <t>176</t>
+  </si>
+  <si>
+    <t>Table B18</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B18.do</t>
+  </si>
+  <si>
+    <t>Table B19</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B19.do</t>
+  </si>
+  <si>
+    <t>240</t>
+  </si>
+  <si>
+    <t>Table B20</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B20.do</t>
+  </si>
+  <si>
+    <t>Table B21</t>
+  </si>
+  <si>
+    <t>code/descriptives/summary_simulation.do</t>
+  </si>
+  <si>
+    <t>29; 72</t>
+  </si>
+  <si>
+    <t>Table B22</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B22.do</t>
+  </si>
+  <si>
+    <t>173</t>
+  </si>
+  <si>
+    <t>Table B23</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B23.do</t>
+  </si>
+  <si>
+    <t>114</t>
+  </si>
+  <si>
+    <t>Table B24</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B24.do</t>
+  </si>
+  <si>
+    <t>Table B25</t>
+  </si>
+  <si>
+    <t>code/descriptives/Table_B25.do</t>
+  </si>
+  <si>
+    <t>Figure B1</t>
+  </si>
+  <si>
+    <t>188</t>
+  </si>
+  <si>
+    <t>Figure B2</t>
+  </si>
+  <si>
+    <t>209</t>
+  </si>
+  <si>
+    <t>Figure B3</t>
+  </si>
+  <si>
+    <t>174</t>
+  </si>
+  <si>
+    <t>Figure B4</t>
+  </si>
+  <si>
+    <t>code/descriptives/gen_omegas_3omegas.do</t>
+  </si>
+  <si>
+    <t>243</t>
+  </si>
+  <si>
+    <t>Figure B5</t>
+  </si>
+  <si>
+    <t>code/descriptives/gen_omegas_tenured.do</t>
+  </si>
+  <si>
+    <t>258</t>
+  </si>
+  <si>
+    <t>Figure B6</t>
+  </si>
+  <si>
+    <t>code/descriptives/gen_omegas_exp1cutoff.do</t>
+  </si>
+  <si>
+    <t>Figure B7</t>
+  </si>
+  <si>
+    <t>code/descriptives/budget_shifts.do</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>Figure B8</t>
+  </si>
+  <si>
+    <t>83; 88; 93; 98</t>
+  </si>
+  <si>
+    <t>Figure B9</t>
+  </si>
+  <si>
+    <t>code/Figure_B9/Figure_B9.do; code/Figure_B9/cutoff_prefs_id_example_graph.R</t>
+  </si>
+  <si>
+    <t>5; 12; 16; 20; 38; 48; 116; 124</t>
+  </si>
+  <si>
+    <t>Figure B10</t>
+  </si>
+  <si>
+    <t>code/descriptives/lambda_map.do</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
     <t>In-text numbers</t>
+  </si>
+  <si>
+    <t>District proficiency ranges: WI 10-80%, CA 10-85%, TX 10-90%</t>
+  </si>
+  <si>
+    <t>Projected Wisconsin budget deficit: $3.6 billion</t>
+  </si>
+  <si>
+    <t>paper p. 7</t>
+  </si>
+  <si>
+    <t>Teachers' share of Wisconsin public employees: 45%</t>
+  </si>
+  <si>
+    <t>Union membership drop: 83% in 2011 to 45% in 2016</t>
+  </si>
+  <si>
+    <t>Wage bounds: 0.3 sd below 1st percentile; 0.2 sd above 99th percentile</t>
+  </si>
+  <si>
+    <t>Student district switching: 4.4% avg.; 4.2/4.3/4.2/4.3% in 2010-2013</t>
+  </si>
+  <si>
+    <t>paper p. 17</t>
+  </si>
+  <si>
+    <t>Non-adopting to adopting district student moves: 0.8/0.8/0.8/0.9% in 2010-2013</t>
+  </si>
+  <si>
+    <t>Public elementary one-school districts: 173 of 411</t>
+  </si>
+  <si>
+    <t>Offer-set identification sample: 5,170 of 6,600 teachers non-singleton</t>
+  </si>
+  <si>
+    <t>Sample exclusions: substitutes 2.0/1.8%; part-time 2.8/3.9% in 2014/2010</t>
+  </si>
+  <si>
+    <t>Experience-correlation with c1/c2: 0.04</t>
+  </si>
+  <si>
+    <t>Observed-vs-predicted wage fit: slope 0.88, se 0.004, R2 0.85; movers slope 1.08, se 0.05, R2 0.75</t>
+  </si>
+  <si>
+    <t>Race controls barely improve Aux 1a R2: 0.680 to 0.681</t>
+  </si>
+  <si>
+    <t>Offer-set robustness shares: 27%, 23%, 21%, 28%</t>
+  </si>
+  <si>
+    <t>Pre-reform wage schedule fit: corr. 0.93; &lt;10% deviation for 95%; slope 0.98, se 0.001, R2 0.99</t>
+  </si>
+  <si>
+    <t>District/school salary R-MSE explanation: 31.3% district FE; 2.7% added school FE</t>
+  </si>
+  <si>
+    <t>Student-composition variation: 8.7% district, +2.7% school, 74% district-level R2; abs. diff mean 0.05, sd 0.06, p25/p50/p75 0.01/0.03/0.07</t>
+  </si>
+  <si>
+    <t>paper p. 13, footnote 12</t>
+  </si>
+  <si>
+    <t>paper p. 2, footnote 1</t>
+  </si>
+  <si>
+    <t>paper p. 17, footnote 17</t>
+  </si>
+  <si>
+    <t>paper p. 6</t>
+  </si>
+  <si>
+    <t>paper p. 19</t>
+  </si>
+  <si>
+    <t>paper p. 24, footnote 30</t>
+  </si>
+  <si>
+    <t>paper p. 27</t>
+  </si>
+  <si>
+    <t>paper p. 27, footnote 34</t>
+  </si>
+  <si>
+    <t>paper p. 28, footnote 35</t>
+  </si>
+  <si>
+    <t>OA p.12</t>
+  </si>
+  <si>
+    <t>OA p.9</t>
+  </si>
+  <si>
+    <t>OA p.18</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -434,19 +1007,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D83"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="111.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59.6640625" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -456,56 +1022,1106 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
+        <v>38</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="D18" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="1"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>2</v>
       </c>
     </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
R2: Issues fixed - One in-text number citation outstanding
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/econ0763/Downloads/JPE/JPE-Biasi-20220349/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8390E1A-4ADB-6640-822D-2BEAB4902A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231E9313-ECE6-6449-B52C-C5F578173245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30240" yWindow="2620" windowWidth="30240" windowHeight="17180" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="197">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -525,9 +525,6 @@
     <t>In-text numbers</t>
   </si>
   <si>
-    <t>District proficiency ranges: WI 10-80%, CA 10-85%, TX 10-90%</t>
-  </si>
-  <si>
     <t>Projected Wisconsin budget deficit: $3.6 billion</t>
   </si>
   <si>
@@ -540,9 +537,6 @@
     <t>Union membership drop: 83% in 2011 to 45% in 2016</t>
   </si>
   <si>
-    <t>Wage bounds: 0.3 sd below 1st percentile; 0.2 sd above 99th percentile</t>
-  </si>
-  <si>
     <t>Student district switching: 4.4% avg.; 4.2/4.3/4.2/4.3% in 2010-2013</t>
   </si>
   <si>
@@ -555,9 +549,6 @@
     <t>Public elementary one-school districts: 173 of 411</t>
   </si>
   <si>
-    <t>Offer-set identification sample: 5,170 of 6,600 teachers non-singleton</t>
-  </si>
-  <si>
     <t>Sample exclusions: substitutes 2.0/1.8%; part-time 2.8/3.9% in 2014/2010</t>
   </si>
   <si>
@@ -582,9 +573,6 @@
     <t>Student-composition variation: 8.7% district, +2.7% school, 74% district-level R2; abs. diff mean 0.05, sd 0.06, p25/p50/p75 0.01/0.03/0.07</t>
   </si>
   <si>
-    <t>paper p. 13, footnote 12</t>
-  </si>
-  <si>
     <t>paper p. 2, footnote 1</t>
   </si>
   <si>
@@ -594,9 +582,6 @@
     <t>paper p. 6</t>
   </si>
   <si>
-    <t>paper p. 19</t>
-  </si>
-  <si>
     <t>paper p. 24, footnote 30</t>
   </si>
   <si>
@@ -619,6 +604,18 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>District proficiency ranges: WI 4-94%, CA 5-89%, TX 6-90%</t>
+  </si>
+  <si>
+    <t>ED Data Express (2021)</t>
+  </si>
+  <si>
+    <t>Wisconsin Taxpayers Alliance (2011)</t>
+  </si>
+  <si>
+    <t>Baron (2018)</t>
   </si>
 </sst>
 </file>
@@ -1007,12 +1004,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D83"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="111.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="59.6640625" customWidth="1"/>
+    <col min="1" max="1" width="83.83203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="36.33203125" customWidth="1"/>
     <col min="3" max="3" width="21.6640625" customWidth="1"/>
+    <col min="4" max="4" width="28.1640625" customWidth="1"/>
+    <col min="5" max="5" width="26.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -1863,13 +1862,13 @@
         <v>32</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" s="1"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>165</v>
       </c>
@@ -1883,242 +1882,215 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="1" t="s">
+      <c r="B68" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C69" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E69" s="2"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B70" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="1" t="s">
-        <v>171</v>
-      </c>
       <c r="B71" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>172</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C72" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D72" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C75" s="2" t="s">
+      <c r="D76" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="D75" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C77" s="2" t="s">
+      <c r="D79" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C80" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="D77" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="D80" s="2" t="s">
-        <v>87</v>
+        <v>32</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>87</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>